<commit_message>
release: prépare la version 0.1.0-snapshot
- sushi-config.yaml : version 0.1.0-snapshot, releaseLabel snapshot
- publication-request.json : version/path/sequence mis à jour, ajout des champs registry
- change-log.md : section 0.1.0-snapshot avec PR #1

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com> 48fe868980d683a97a55f8c0822f7bb461c6804e
</commit_message>
<xml_diff>
--- a/release/0.1.0-snapshot/ig/StructureDefinition-as-bal-mss-app.xlsx
+++ b/release/0.1.0-snapshot/ig/StructureDefinition-as-bal-mss-app.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.1.0</t>
+    <t>0.1.0-snapshot</t>
   </si>
   <si>
     <t>Name</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-18T15:43:12+00:00</t>
+    <t>2026-06-18T15:49:17+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>